<commit_message>
002 2.1: columnas del eje 3 en HSST10X6X0.188 (medida par)
El HSS 9x9 no existe comercialmente; el HSST10X6X0.188 es el HSS de medidas
pares mas ligero que pasa (mismo peso que el 8x8x3/16, con mas holgura en
flecha). Factores X 1.1213 / Z 1.4625, CUT OFF 42. 7470.6 kg, 48.64 kg/m2
con 5% de conexiones. Desglose y hoja de sismo actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DbpSpoM7qi5cJ9LMKpwgVv
</commit_message>
<xml_diff>
--- a/002/002_SISMO_VIENTO_SALVADOR_2.1.xlsx
+++ b/002/002_SISMO_VIENTO_SALVADOR_2.1.xlsx
@@ -6480,7 +6480,7 @@
         <v>68</v>
       </c>
       <c r="F137" s="36">
-        <v>0.69136</v>
+        <v>0.69385</v>
       </c>
       <c r="G137" t="s">
         <v>66</v>
@@ -6492,7 +6492,7 @@
       </c>
       <c r="F139" s="52">
         <f>P33*Q85*P55/P99*(P57/MAX(P57,MIN(F137,6*P57)))^(2/3)</f>
-        <v>0.155972442667178</v>
+        <v>0.155599063172964</v>
       </c>
     </row>
     <row r="140" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="F143" s="54">
         <f>MAX(F141,F139)</f>
-        <v>0.155972442667178</v>
+        <v>0.155599063172964</v>
       </c>
     </row>
     <row r="148" spans="2:25" s="39" customFormat="1" x14ac:dyDescent="0.3"/>
@@ -6635,14 +6635,14 @@
         <v>87</v>
       </c>
       <c r="E165" s="82">
-        <v>13076.56</v>
+        <v>13196.88</v>
       </c>
       <c r="F165" s="1" t="s">
         <v>85</v>
       </c>
       <c r="G165" s="55">
         <f>E165/1000</f>
-        <v>13.07656</v>
+        <v>13.19688</v>
       </c>
       <c r="H165" s="1" t="s">
         <v>86</v>
@@ -6653,14 +6653,14 @@
         <v>88</v>
       </c>
       <c r="E166" s="82">
-        <v>13076.56</v>
+        <v>13196.88</v>
       </c>
       <c r="F166" s="1" t="s">
         <v>85</v>
       </c>
       <c r="G166" s="55">
         <f>E166/1000</f>
-        <v>13.07656</v>
+        <v>13.19688</v>
       </c>
       <c r="H166" s="1" t="s">
         <v>86</v>
@@ -6697,7 +6697,7 @@
       </c>
       <c r="G170" s="51">
         <f>G168*G165</f>
-        <v>2.241696</v>
+        <v>2.26232228571429</v>
       </c>
       <c r="H170" s="1" t="s">
         <v>86</v>
@@ -6714,7 +6714,7 @@
       </c>
       <c r="G171" s="51">
         <f>G168*G166</f>
-        <v>2.241696</v>
+        <v>2.26232228571429</v>
       </c>
       <c r="H171" s="1" t="s">
         <v>86</v>
@@ -6826,13 +6826,13 @@
         <v>1</v>
       </c>
       <c r="C177" s="28">
-        <v>1.446</v>
+        <v>1.441</v>
       </c>
       <c r="D177" s="64">
-        <v>0.69136</v>
+        <v>0.69385</v>
       </c>
       <c r="E177" s="28">
-        <v>80.18</v>
+        <v>80.02</v>
       </c>
       <c r="F177" s="28">
         <v>0</v>
@@ -6853,7 +6853,7 @@
       </c>
       <c r="K177" s="32">
         <f>J177*$K$221*E177/100</f>
-        <v>1637.48579750817</v>
+        <v>1649.25494087403</v>
       </c>
       <c r="L177" s="34">
         <f>J177*$K$222*G177/100</f>
@@ -6875,13 +6875,13 @@
         <v>2</v>
       </c>
       <c r="C178" s="28">
-        <v>2.682</v>
+        <v>2.68</v>
       </c>
       <c r="D178" s="64">
-        <v>0.37285</v>
+        <v>0.37312</v>
       </c>
       <c r="E178" s="28">
-        <v>0.01</v>
+        <v>5.39</v>
       </c>
       <c r="F178" s="28">
         <v>0</v>
@@ -6902,7 +6902,7 @@
       </c>
       <c r="K178" s="32">
         <f>J178*$K$221*E178/100</f>
-        <v>0.2241696</v>
+        <v>121.9391712</v>
       </c>
       <c r="L178" s="34">
         <f>J178*$K$222*G178/100</f>
@@ -6965,13 +6965,13 @@
         <v>4</v>
       </c>
       <c r="C180" s="28">
-        <v>2.689</v>
+        <v>2.682</v>
       </c>
       <c r="D180" s="64">
-        <v>0.3719</v>
+        <v>0.37285</v>
       </c>
       <c r="E180" s="28">
-        <v>5.37</v>
+        <v>0.01</v>
       </c>
       <c r="F180" s="28">
         <v>0</v>
@@ -6992,7 +6992,7 @@
       </c>
       <c r="K180" s="32">
         <f t="shared" ref="K180:K218" si="7">J180*$K$221*E180/100</f>
-        <v>120.3790752</v>
+        <v>0.226232228571429</v>
       </c>
       <c r="L180" s="34">
         <f t="shared" ref="L180:L218" si="8">J180*$K$222*G180/100</f>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="K182" s="32">
         <f t="shared" si="7"/>
-        <v>0.4483392</v>
+        <v>0.452464457142857</v>
       </c>
       <c r="L182" s="34">
         <f t="shared" si="8"/>
@@ -7088,10 +7088,10 @@
         <v>7</v>
       </c>
       <c r="C183" s="28">
-        <v>3.323</v>
+        <v>3.319</v>
       </c>
       <c r="D183" s="64">
-        <v>0.3009</v>
+        <v>0.30132</v>
       </c>
       <c r="E183" s="28">
         <v>0</v>
@@ -7100,7 +7100,7 @@
         <v>0</v>
       </c>
       <c r="G183" s="28">
-        <v>57.3</v>
+        <v>57.6</v>
       </c>
       <c r="H183" s="28" t="s">
         <v>113</v>
@@ -7119,7 +7119,7 @@
       </c>
       <c r="L183" s="34">
         <f t="shared" si="8"/>
-        <v>1284.491808</v>
+        <v>1303.09763657143</v>
       </c>
       <c r="N183" s="10"/>
       <c r="O183" s="26"/>
@@ -7129,13 +7129,13 @@
         <v>8</v>
       </c>
       <c r="C184" s="28">
-        <v>4.2</v>
+        <v>4.199</v>
       </c>
       <c r="D184" s="64">
-        <v>0.23812</v>
+        <v>0.23814</v>
       </c>
       <c r="E184" s="28">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="F184" s="28">
         <v>0</v>
@@ -7156,7 +7156,7 @@
       </c>
       <c r="K184" s="32">
         <f t="shared" si="7"/>
-        <v>10.7601408</v>
+        <v>10.6329147428571</v>
       </c>
       <c r="L184" s="34">
         <f t="shared" si="8"/>
@@ -7170,10 +7170,10 @@
         <v>9</v>
       </c>
       <c r="C185" s="28">
-        <v>4.302</v>
+        <v>4.296</v>
       </c>
       <c r="D185" s="64">
-        <v>0.23247</v>
+        <v>0.23279</v>
       </c>
       <c r="E185" s="28">
         <v>0</v>
@@ -7182,7 +7182,7 @@
         <v>0</v>
       </c>
       <c r="G185" s="28">
-        <v>16.22</v>
+        <v>16.34</v>
       </c>
       <c r="H185" s="28" t="s">
         <v>113</v>
@@ -7201,7 +7201,7 @@
       </c>
       <c r="L185" s="34">
         <f t="shared" si="8"/>
-        <v>363.6030912</v>
+        <v>369.663461485714</v>
       </c>
       <c r="N185" s="10"/>
     </row>
@@ -7292,10 +7292,10 @@
         <v>12</v>
       </c>
       <c r="C188" s="28">
-        <v>4.688</v>
+        <v>4.683</v>
       </c>
       <c r="D188" s="64">
-        <v>0.21329</v>
+        <v>0.21355</v>
       </c>
       <c r="E188" s="28">
         <v>0</v>
@@ -7304,7 +7304,7 @@
         <v>0</v>
       </c>
       <c r="G188" s="28">
-        <v>14.55</v>
+        <v>14.04</v>
       </c>
       <c r="H188" s="28" t="s">
         <v>113</v>
@@ -7323,7 +7323,7 @@
       </c>
       <c r="L188" s="34">
         <f t="shared" si="8"/>
-        <v>326.166768</v>
+        <v>317.630048914286</v>
       </c>
       <c r="N188" s="10" t="s">
         <v>114</v>
@@ -7493,10 +7493,10 @@
         <v>15</v>
       </c>
       <c r="C191" s="28">
-        <v>6.624</v>
+        <v>7.039</v>
       </c>
       <c r="D191" s="64">
-        <v>0.15096</v>
+        <v>0.14207</v>
       </c>
       <c r="E191" s="28">
         <v>0</v>
@@ -7512,11 +7512,11 @@
       </c>
       <c r="I191" s="29">
         <f t="shared" si="5"/>
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="J191" s="31">
         <f t="shared" si="6"/>
-        <v>0.142857142857143</v>
+        <v>0.137142857142857</v>
       </c>
       <c r="K191" s="32">
         <f t="shared" si="7"/>
@@ -7557,13 +7557,13 @@
         <v>16</v>
       </c>
       <c r="C192" s="28">
-        <v>6.804</v>
+        <v>7.081</v>
       </c>
       <c r="D192" s="64">
-        <v>0.14697</v>
+        <v>0.14122</v>
       </c>
       <c r="E192" s="28">
-        <v>1.16</v>
+        <v>0.29</v>
       </c>
       <c r="F192" s="28">
         <v>0</v>
@@ -7576,15 +7576,15 @@
       </c>
       <c r="I192" s="29">
         <f t="shared" si="5"/>
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="J192" s="31">
         <f t="shared" si="6"/>
-        <v>0.142857142857143</v>
+        <v>0.137142857142857</v>
       </c>
       <c r="K192" s="32">
         <f t="shared" si="7"/>
-        <v>21.669728</v>
+        <v>5.24858770285714</v>
       </c>
       <c r="L192" s="34">
         <f t="shared" si="8"/>
@@ -7621,13 +7621,13 @@
         <v>17</v>
       </c>
       <c r="C193" s="28">
-        <v>7.118</v>
+        <v>7.14</v>
       </c>
       <c r="D193" s="64">
-        <v>0.1405</v>
+        <v>0.14006</v>
       </c>
       <c r="E193" s="28">
-        <v>0.16</v>
+        <v>0.9</v>
       </c>
       <c r="F193" s="28">
         <v>0</v>
@@ -7648,7 +7648,7 @@
       </c>
       <c r="K193" s="32">
         <f t="shared" si="7"/>
-        <v>2.86937088</v>
+        <v>16.2887204571429</v>
       </c>
       <c r="L193" s="34">
         <f t="shared" si="8"/>
@@ -7810,10 +7810,10 @@
         <v>20</v>
       </c>
       <c r="C196" s="28">
-        <v>7.37</v>
+        <v>7.377</v>
       </c>
       <c r="D196" s="64">
-        <v>0.13568</v>
+        <v>0.13556</v>
       </c>
       <c r="E196" s="28">
         <v>0</v>
@@ -7873,10 +7873,10 @@
         <v>21</v>
       </c>
       <c r="C197" s="28">
-        <v>7.408</v>
+        <v>7.405</v>
       </c>
       <c r="D197" s="64">
-        <v>0.13499</v>
+        <v>0.13504</v>
       </c>
       <c r="E197" s="28">
         <v>0</v>
@@ -7892,11 +7892,11 @@
       </c>
       <c r="I197" s="29">
         <f t="shared" si="5"/>
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="J197" s="31">
         <f t="shared" si="6"/>
-        <v>0.131428571428571</v>
+        <v>0.137142857142857</v>
       </c>
       <c r="K197" s="32">
         <f t="shared" si="7"/>
@@ -7936,13 +7936,13 @@
         <v>22</v>
       </c>
       <c r="C198" s="28">
-        <v>7.429</v>
+        <v>7.428</v>
       </c>
       <c r="D198" s="64">
-        <v>0.13461</v>
+        <v>0.13463</v>
       </c>
       <c r="E198" s="28">
-        <v>1.94</v>
+        <v>2.11</v>
       </c>
       <c r="F198" s="28">
         <v>0</v>
@@ -7963,7 +7963,7 @@
       </c>
       <c r="K198" s="32">
         <f t="shared" si="7"/>
-        <v>33.34149184</v>
+        <v>36.5968335085714</v>
       </c>
       <c r="L198" s="34">
         <f t="shared" si="8"/>
@@ -7999,10 +7999,10 @@
         <v>23</v>
       </c>
       <c r="C199" s="28">
-        <v>7.499</v>
+        <v>7.498</v>
       </c>
       <c r="D199" s="64">
-        <v>0.13335</v>
+        <v>0.13336</v>
       </c>
       <c r="E199" s="28">
         <v>0</v>
@@ -8030,7 +8030,7 @@
       </c>
       <c r="L199" s="34">
         <f t="shared" si="8"/>
-        <v>1.03118016</v>
+        <v>1.04066825142857</v>
       </c>
       <c r="T199">
         <v>12</v>
@@ -8125,13 +8125,13 @@
         <v>25</v>
       </c>
       <c r="C201" s="28">
-        <v>7.565</v>
+        <v>7.566</v>
       </c>
       <c r="D201" s="64">
-        <v>0.13219</v>
+        <v>0.13217</v>
       </c>
       <c r="E201" s="28">
-        <v>0.35</v>
+        <v>0.32</v>
       </c>
       <c r="F201" s="28">
         <v>0</v>
@@ -8152,7 +8152,7 @@
       </c>
       <c r="K201" s="32">
         <f t="shared" si="7"/>
-        <v>6.0152176</v>
+        <v>5.55023067428571</v>
       </c>
       <c r="L201" s="34">
         <f t="shared" si="8"/>
@@ -8257,7 +8257,7 @@
         <v>0.13181</v>
       </c>
       <c r="E203" s="28">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="F203" s="28">
         <v>0</v>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="K203" s="32">
         <f t="shared" si="7"/>
-        <v>4.296584</v>
+        <v>4.50956242285714</v>
       </c>
       <c r="L203" s="34">
         <f t="shared" si="8"/>
@@ -8378,13 +8378,13 @@
         <v>29</v>
       </c>
       <c r="C205" s="28">
-        <v>7.593</v>
+        <v>7.594</v>
       </c>
       <c r="D205" s="64">
         <v>0.13169</v>
       </c>
       <c r="E205" s="28">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="F205" s="28">
         <v>0</v>
@@ -8405,7 +8405,7 @@
       </c>
       <c r="K205" s="32">
         <f t="shared" si="7"/>
-        <v>0.8593168</v>
+        <v>0.693778834285714</v>
       </c>
       <c r="L205" s="34">
         <f t="shared" si="8"/>
@@ -8531,7 +8531,7 @@
       </c>
       <c r="K207" s="32">
         <f t="shared" si="7"/>
-        <v>0.51559008</v>
+        <v>0.520334125714286</v>
       </c>
       <c r="L207" s="34">
         <f t="shared" si="8"/>
@@ -8756,13 +8756,13 @@
         <v>35</v>
       </c>
       <c r="C211" s="28">
-        <v>7.647</v>
+        <v>7.65</v>
       </c>
       <c r="D211" s="64">
-        <v>0.13077</v>
+        <v>0.13072</v>
       </c>
       <c r="E211" s="28">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="F211" s="28">
         <v>0</v>
@@ -8783,7 +8783,7 @@
       </c>
       <c r="K211" s="32">
         <f t="shared" si="7"/>
-        <v>0.34372672</v>
+        <v>0.693778834285714</v>
       </c>
       <c r="L211" s="34">
         <f t="shared" si="8"/>
@@ -8846,7 +8846,7 @@
       </c>
       <c r="K212" s="32">
         <f t="shared" si="7"/>
-        <v>7.7338512</v>
+        <v>7.80501188571429</v>
       </c>
       <c r="L212" s="34">
         <f t="shared" si="8"/>
@@ -8909,7 +8909,7 @@
       </c>
       <c r="K213" s="32">
         <f t="shared" si="7"/>
-        <v>7.04639776</v>
+        <v>7.11123305142857</v>
       </c>
       <c r="L213" s="34">
         <f t="shared" si="8"/>
@@ -8945,13 +8945,13 @@
         <v>38</v>
       </c>
       <c r="C214" s="28">
-        <v>8.177</v>
+        <v>8.185</v>
       </c>
       <c r="D214" s="64">
-        <v>0.12229</v>
+        <v>0.12218</v>
       </c>
       <c r="E214" s="28">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="F214" s="28">
         <v>0</v>
@@ -8972,7 +8972,7 @@
       </c>
       <c r="K214" s="32">
         <f t="shared" si="7"/>
-        <v>0.16439104</v>
+        <v>0.497710902857143</v>
       </c>
       <c r="L214" s="34">
         <f t="shared" si="8"/>
@@ -9008,19 +9008,19 @@
         <v>39</v>
       </c>
       <c r="C215" s="28">
-        <v>9.307</v>
+        <v>9.274</v>
       </c>
       <c r="D215" s="64">
-        <v>0.10745</v>
+        <v>0.10783</v>
       </c>
       <c r="E215" s="28">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="F215" s="28">
         <v>0</v>
       </c>
       <c r="G215" s="28">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="H215" s="28" t="s">
         <v>113</v>
@@ -9035,11 +9035,11 @@
       </c>
       <c r="K215" s="32">
         <f t="shared" si="7"/>
-        <v>0.15691872</v>
+        <v>0.31672512</v>
       </c>
       <c r="L215" s="34">
         <f t="shared" si="8"/>
-        <v>0.62767488</v>
+        <v>0.7918128</v>
       </c>
       <c r="T215">
         <v>30</v>
@@ -9071,19 +9071,19 @@
         <v>40</v>
       </c>
       <c r="C216" s="28">
-        <v>10.102</v>
+        <v>10.051</v>
       </c>
       <c r="D216" s="64">
-        <v>0.09899</v>
+        <v>0.09949</v>
       </c>
       <c r="E216" s="28">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="F216" s="28">
         <v>0</v>
       </c>
       <c r="G216" s="28">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="H216" s="28" t="s">
         <v>113</v>
@@ -9098,11 +9098,11 @@
       </c>
       <c r="K216" s="32">
         <f t="shared" si="7"/>
-        <v>0.5977856</v>
+        <v>0.150821485714286</v>
       </c>
       <c r="L216" s="34">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>7.69189577142857</v>
       </c>
       <c r="T216">
         <v>31</v>
@@ -9134,19 +9134,19 @@
         <v>41</v>
       </c>
       <c r="C217" s="28">
-        <v>10.249</v>
+        <v>10.125</v>
       </c>
       <c r="D217" s="64">
-        <v>0.09757</v>
+        <v>0.09877</v>
       </c>
       <c r="E217" s="28">
-        <v>0.09</v>
+        <v>0.02</v>
       </c>
       <c r="F217" s="28">
         <v>0</v>
       </c>
       <c r="G217" s="28">
-        <v>0.07</v>
+        <v>3.2</v>
       </c>
       <c r="H217" s="28" t="s">
         <v>113</v>
@@ -9161,11 +9161,11 @@
       </c>
       <c r="K217" s="32">
         <f t="shared" si="7"/>
-        <v>1.3450176</v>
+        <v>0.301642971428571</v>
       </c>
       <c r="L217" s="34">
         <f t="shared" si="8"/>
-        <v>1.0461248</v>
+        <v>48.2628754285714</v>
       </c>
       <c r="T217">
         <v>32</v>
@@ -9197,19 +9197,19 @@
         <v>42</v>
       </c>
       <c r="C218" s="28">
-        <v>10.455</v>
+        <v>10.155</v>
       </c>
       <c r="D218" s="64">
-        <v>0.09564</v>
+        <v>0.09847</v>
       </c>
       <c r="E218" s="28">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="F218" s="28">
         <v>0</v>
       </c>
       <c r="G218" s="28">
-        <v>4.46</v>
+        <v>0.78</v>
       </c>
       <c r="H218" s="28" t="s">
         <v>113</v>
@@ -9224,11 +9224,11 @@
       </c>
       <c r="K218" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.80985782857143</v>
       </c>
       <c r="L218" s="34">
         <f t="shared" si="8"/>
-        <v>66.6530944</v>
+        <v>11.7640758857143</v>
       </c>
       <c r="T218">
         <v>50</v>
@@ -9263,7 +9263,7 @@
       <c r="D219" s="115"/>
       <c r="E219" s="116">
         <f>SUM(E177:E218)</f>
-        <v>91.03</v>
+        <v>90.96</v>
       </c>
       <c r="F219" s="116">
         <f t="shared" ref="F219" si="9">SUM(F177:F218)</f>
@@ -9271,7 +9271,7 @@
       </c>
       <c r="G219" s="116">
         <f>SUM(G177:G218)</f>
-        <v>92.7</v>
+        <v>92.58</v>
       </c>
       <c r="H219" s="140" t="s">
         <v>131</v>
@@ -9280,11 +9280,11 @@
       <c r="J219" s="142"/>
       <c r="K219" s="117">
         <f>SQRT(SUMSQ(K177:K218))</f>
-        <v>1642.47490217752</v>
+        <v>1654.33495229314</v>
       </c>
       <c r="L219" s="117">
         <f>SQRT(SUMSQ(L177:L218))</f>
-        <v>1375.84750607592</v>
+        <v>1392.16807426887</v>
       </c>
       <c r="T219">
         <v>51</v>
@@ -9346,7 +9346,7 @@
       </c>
       <c r="K221" s="30">
         <f>E165</f>
-        <v>13076.56</v>
+        <v>13196.88</v>
       </c>
       <c r="L221" t="s">
         <v>134</v>
@@ -9385,7 +9385,7 @@
       </c>
       <c r="K222" s="30">
         <f>E166</f>
-        <v>13076.56</v>
+        <v>13196.88</v>
       </c>
       <c r="L222" t="s">
         <v>134</v>
@@ -9452,11 +9452,11 @@
       </c>
       <c r="K224" s="30">
         <f>K221*VLOOKUP(MAX(E177:E218),E177:J218,6,0)</f>
-        <v>2042.26215703189</v>
+        <v>2061.05341273936</v>
       </c>
       <c r="L224" s="30">
         <f>K221*VLOOKUP(MAX(G177:G218),G177:J218,4,0)</f>
-        <v>2241.696</v>
+        <v>2262.32228571429</v>
       </c>
       <c r="T224">
         <v>56</v>
@@ -9489,11 +9489,11 @@
       </c>
       <c r="K225" s="30">
         <f>0.9*K224</f>
-        <v>1838.0359413287</v>
+        <v>1854.94807146542</v>
       </c>
       <c r="L225" s="30">
         <f>0.9*L224</f>
-        <v>2017.5264</v>
+        <v>2036.09005714286</v>
       </c>
       <c r="T225">
         <v>57</v>
@@ -9558,11 +9558,11 @@
       </c>
       <c r="K227" s="30">
         <f>K221*G168</f>
-        <v>2241.696</v>
+        <v>2262.32228571429</v>
       </c>
       <c r="L227" s="30">
         <f>K221*G168</f>
-        <v>2241.696</v>
+        <v>2262.32228571429</v>
       </c>
       <c r="T227">
         <v>59</v>
@@ -9595,11 +9595,11 @@
       </c>
       <c r="K228" s="30">
         <f>0.8*K227</f>
-        <v>1793.3568</v>
+        <v>1809.85782857143</v>
       </c>
       <c r="L228" s="30">
         <f>0.8*L227</f>
-        <v>1793.3568</v>
+        <v>1809.85782857143</v>
       </c>
       <c r="T228">
         <v>60</v>
@@ -9688,11 +9688,11 @@
       </c>
       <c r="K231" s="44">
         <f>MAX(K228,K225)</f>
-        <v>1838.0359413287</v>
+        <v>1854.94807146542</v>
       </c>
       <c r="L231" s="44">
         <f>MAX(L228,L225)</f>
-        <v>2017.5264</v>
+        <v>2036.09005714286</v>
       </c>
       <c r="T231">
         <v>63</v>
@@ -9814,11 +9814,11 @@
       </c>
       <c r="K235" s="47">
         <f>K231/1000</f>
-        <v>1.8380359413287</v>
+        <v>1.85494807146542</v>
       </c>
       <c r="L235" s="47">
         <f>L231/1000</f>
-        <v>2.0175264</v>
+        <v>2.03609005714286</v>
       </c>
       <c r="T235">
         <v>67</v>
@@ -9851,11 +9851,11 @@
       </c>
       <c r="K236" s="47">
         <f>K219/1000</f>
-        <v>1.64247490217752</v>
+        <v>1.65433495229314</v>
       </c>
       <c r="L236" s="47">
         <f>L219/1000</f>
-        <v>1.37584750607592</v>
+        <v>1.39216807426887</v>
       </c>
       <c r="T236">
         <v>68</v>
@@ -9925,11 +9925,11 @@
       </c>
       <c r="K238" s="86">
         <f>MAX(K235/K236,1)</f>
-        <v>1.1190648568766</v>
+        <v>1.12126511556454</v>
       </c>
       <c r="L238" s="86">
         <f>MAX(L235/L236,1)</f>
-        <v>1.46638809249596</v>
+        <v>1.46253178389553</v>
       </c>
       <c r="T238">
         <v>70</v>
@@ -9988,11 +9988,11 @@
       </c>
       <c r="K240" s="86">
         <f>IF(K225/K219&lt;1,"N/A",K225/K219)</f>
-        <v>1.1190648568766</v>
+        <v>1.12126511556454</v>
       </c>
       <c r="L240" s="86">
         <f>IF(L225/L219&lt;1,"N/A",L225/L219)</f>
-        <v>1.46638809249596</v>
+        <v>1.46253178389553</v>
       </c>
       <c r="T240">
         <v>72</v>
@@ -10048,11 +10048,11 @@
     <row r="242" spans="2:27" x14ac:dyDescent="0.3">
       <c r="K242" s="53">
         <f>K224/K219</f>
-        <v>1.24340539652956</v>
+        <v>1.24585012840505</v>
       </c>
       <c r="L242" s="53">
         <f>L224/L219</f>
-        <v>1.62932010277329</v>
+        <v>1.62503531543948</v>
       </c>
       <c r="T242">
         <v>74</v>

</xml_diff>